<commit_message>
Fix tab defaults, template downloads, and xlsx import templates
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/client-dist/templates/PriceRight_Materials_Import_Template.xlsx
+++ b/client-dist/templates/PriceRight_Materials_Import_Template.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Materials Import" sheetId="1" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="1" r:id="rId1"/>
+    <sheet name="Import Data" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +398,90 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:A12"/>
+  <cols>
+    <col min="1" max="1" width="100.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Primary Materials Import Template</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Fill in your materials on the Import Data sheet.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Each row is one material.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Required columns: Material Name, Category, Unit, Bulk Price, Bulk Quantity.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Optional columns: Purchase Currency (defaults to base currency GHS), Supplier Type (Local or Foreign).</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Currency Code must match a currency configured in PriceRight Settings (GHS, USD, EUR, etc.).</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Leave Purchase Currency blank to use the base currency (GHS).</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>After filling in the template, save as CSV (File → Save As → CSV UTF-8) and upload in the import dialog.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A12"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G1"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="19.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,55 +506,9 @@
         <v>Supplier Type</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Bottle Tray - Honey 400g</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Packaging</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Ea</v>
-      </c>
-      <c r="D2" t="str">
-        <v>GHS</v>
-      </c>
-      <c r="E2">
-        <v>25</v>
-      </c>
-      <c r="F2">
-        <v>50</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Local</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Sugar</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Ingredients</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D3" t="str">
-        <v>USD</v>
-      </c>
-      <c r="E3">
-        <v>320.5</v>
-      </c>
-      <c r="F3">
-        <v>25</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Foreign</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve import templates — numbered instructions, column guide with examples, sample data rows, delete-before-import note
</commit_message>
<xml_diff>
--- a/client-dist/templates/PriceRight_Materials_Import_Template.xlsx
+++ b/client-dist/templates/PriceRight_Materials_Import_Template.xlsx
@@ -398,14 +398,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A61"/>
   <cols>
     <col min="1" max="1" width="100.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Primary Materials Import Template</v>
+        <v>PriceRight — Materials Import Template</v>
       </c>
     </row>
     <row r="2">
@@ -415,72 +415,319 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Fill in your materials on the Import Data sheet.</v>
+        <v>HOW TO USE THIS TEMPLATE</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Each row is one material.</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v/>
+        <v>STEPS:</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Required columns: Material Name, Category, Unit, Bulk Price, Bulk Quantity.</v>
+        <v>1. Click the "Import Data" tab at the bottom of this file</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Optional columns: Purchase Currency (defaults to base currency GHS), Supplier Type (Local or Foreign).</v>
+        <v>2. Review the sample rows to understand the expected format</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v>3. Delete the sample data rows (rows 2 and below)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Currency Code must match a currency configured in PriceRight Settings (GHS, USD, EUR, etc.).</v>
+        <v xml:space="preserve">   — Keep row 1 (the column headers) — do not delete or edit it</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Leave Purchase Currency blank to use the base currency (GHS).</v>
+        <v>4. Enter your real data starting from row 2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>5. Save the file (keep the .xlsx format)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>After filling in the template, save as CSV (File → Save As → CSV UTF-8) and upload in the import dialog.</v>
+        <v>6. In PriceRight go to Materials → More → Import and select this file</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>IMPORTANT NOTES:</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>— Do not rename or delete any column headers</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>— Do not add extra columns</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>— Leave optional fields blank if not needed</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>— Currency codes must match currencies set up in PriceRight</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>COLUMN GUIDE:</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v xml:space="preserve">  Material Name — Required</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v xml:space="preserve">    The full name of the raw material as it will appear in PriceRight</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v xml:space="preserve">    Example: Cocoa Beans (Dried)</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v xml:space="preserve">  SKU — Optional</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v xml:space="preserve">    Your internal stock keeping unit or product code</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v xml:space="preserve">    Example: RM-001</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v xml:space="preserve">  Category — Required</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v xml:space="preserve">    The material category. Must match a category in PriceRight</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v xml:space="preserve">    or a new one will be created automatically</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v xml:space="preserve">    Example: Cocoa</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v xml:space="preserve">  Unit — Required</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v xml:space="preserve">    Unit of measure for this material</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v xml:space="preserve">    Example: Kg   L   Ea   m   g</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v xml:space="preserve">  Supplier — Optional</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v xml:space="preserve">    Name of the supplier for this material</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v xml:space="preserve">    Example: Agro Distributors Ltd</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v xml:space="preserve">  Bulk Price — Required</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v xml:space="preserve">    The price paid for the bulk quantity below</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v xml:space="preserve">    Example: 562.50</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v xml:space="preserve">  Bulk Quantity — Required</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v xml:space="preserve">    The quantity the bulk price applies to</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v xml:space="preserve">    Example: 25  (meaning GHS 562.50 for 25 Kg)</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v xml:space="preserve">  Currency Code — Required</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v xml:space="preserve">    The currency of purchase. Must be set up in PriceRight first</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v xml:space="preserve">    Example: GHS   USD   EUR</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v xml:space="preserve">  Description — Optional</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v xml:space="preserve">    Any additional notes about this material</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v xml:space="preserve">    Example: Premium grade sun-dried cocoa beans</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>SAMPLE DATA:</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>The Import Data sheet contains sample rows showing the correct format.</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Delete them before importing.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A61"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I4"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="19.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,27 +735,120 @@
         <v>Material Name</v>
       </c>
       <c r="B1" t="str">
+        <v>SKU</v>
+      </c>
+      <c r="C1" t="str">
         <v>Category</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Unit</v>
       </c>
-      <c r="D1" t="str">
-        <v>Purchase Currency</v>
-      </c>
       <c r="E1" t="str">
+        <v>Supplier</v>
+      </c>
+      <c r="F1" t="str">
         <v>Bulk Price</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Bulk Quantity</v>
       </c>
-      <c r="G1" t="str">
-        <v>Supplier Type</v>
+      <c r="H1" t="str">
+        <v>Currency Code</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Description</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Cocoa Beans (Dried)</v>
+      </c>
+      <c r="B2" t="str">
+        <v>RM-001</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Cocoa</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Agro Distributors Ltd</v>
+      </c>
+      <c r="F2">
+        <v>562.5</v>
+      </c>
+      <c r="G2">
+        <v>25</v>
+      </c>
+      <c r="H2" t="str">
+        <v>GHS</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Premium grade sun-dried cocoa beans</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Palm Oil (Crude)</v>
+      </c>
+      <c r="B3" t="str">
+        <v>RM-002</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Oils &amp; Fats</v>
+      </c>
+      <c r="D3" t="str">
+        <v>L</v>
+      </c>
+      <c r="E3" t="str">
+        <v>West Africa Oils</v>
+      </c>
+      <c r="F3">
+        <v>187.5</v>
+      </c>
+      <c r="G3">
+        <v>25</v>
+      </c>
+      <c r="H3" t="str">
+        <v>GHS</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Refined palm oil for food production</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Packaging Film (Roll)</v>
+      </c>
+      <c r="B4" t="str">
+        <v>RM-003</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Packaging</v>
+      </c>
+      <c r="D4" t="str">
+        <v>m</v>
+      </c>
+      <c r="E4" t="str">
+        <v>PackRight Ltd</v>
+      </c>
+      <c r="F4">
+        <v>850</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4" t="str">
+        <v>GHS</v>
+      </c>
+      <c r="I4" t="str">
+        <v>100m roll of clear heat-seal packaging film</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Bump to v1.0.12: intermediate materials fixes, supplier simplification, tab styling, PR branding
Fix intermediate material edit navigation and dashboard stats. Remove supplier from UI and import templates. Add vivid section and choice tab styling. Add PR sidebar icon and logo assets.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/client-dist/templates/PriceRight_Materials_Import_Template.xlsx
+++ b/client-dist/templates/PriceRight_Materials_Import_Template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A61"/>
+  <dimension ref="A1:A57"/>
   <cols>
     <col min="1" max="1" width="100.83203125" customWidth="1"/>
   </cols>
@@ -595,17 +595,17 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v xml:space="preserve">  Supplier — Optional</v>
+        <v xml:space="preserve">  Bulk Price — Required</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v xml:space="preserve">    Name of the supplier for this material</v>
+        <v xml:space="preserve">    The price paid for the bulk quantity below</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v xml:space="preserve">    Example: Agro Distributors Ltd</v>
+        <v xml:space="preserve">    Example: 562.50</v>
       </c>
     </row>
     <row r="42">
@@ -615,17 +615,17 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v xml:space="preserve">  Bulk Price — Required</v>
+        <v xml:space="preserve">  Bulk Quantity — Required</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v xml:space="preserve">    The price paid for the bulk quantity below</v>
+        <v xml:space="preserve">    The quantity the bulk price applies to</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v xml:space="preserve">    Example: 562.50</v>
+        <v xml:space="preserve">    Example: 25  (meaning GHS 562.50 for 25 Kg)</v>
       </c>
     </row>
     <row r="46">
@@ -635,17 +635,17 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v xml:space="preserve">  Bulk Quantity — Required</v>
+        <v xml:space="preserve">  Currency Code — Required</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v xml:space="preserve">    The quantity the bulk price applies to</v>
+        <v xml:space="preserve">    The currency of purchase. Must be set up in PriceRight first</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v xml:space="preserve">    Example: 25  (meaning GHS 562.50 for 25 Kg)</v>
+        <v xml:space="preserve">    Example: GHS   USD   EUR</v>
       </c>
     </row>
     <row r="50">
@@ -655,17 +655,17 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v xml:space="preserve">  Currency Code — Required</v>
+        <v xml:space="preserve">  Description — Optional</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v xml:space="preserve">    The currency of purchase. Must be set up in PriceRight first</v>
+        <v xml:space="preserve">    Any additional notes about this material</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v xml:space="preserve">    Example: GHS   USD   EUR</v>
+        <v xml:space="preserve">    Example: Premium grade sun-dried cocoa beans</v>
       </c>
     </row>
     <row r="54">
@@ -675,49 +675,29 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v xml:space="preserve">  Description — Optional</v>
+        <v>SAMPLE DATA:</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v xml:space="preserve">    Any additional notes about this material</v>
+        <v>The Import Data sheet contains sample rows showing the correct format.</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v xml:space="preserve">    Example: Premium grade sun-dried cocoa beans</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>SAMPLE DATA:</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v>The Import Data sheet contains sample rows showing the correct format.</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="str">
         <v>Delete them before importing.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A57"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:H4"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -727,7 +707,6 @@
     <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="18.83203125" customWidth="1"/>
     <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -744,18 +723,15 @@
         <v>Unit</v>
       </c>
       <c r="E1" t="str">
-        <v>Supplier</v>
+        <v>Bulk Price</v>
       </c>
       <c r="F1" t="str">
-        <v>Bulk Price</v>
+        <v>Bulk Quantity</v>
       </c>
       <c r="G1" t="str">
-        <v>Bulk Quantity</v>
+        <v>Currency Code</v>
       </c>
       <c r="H1" t="str">
-        <v>Currency Code</v>
-      </c>
-      <c r="I1" t="str">
         <v>Description</v>
       </c>
     </row>
@@ -772,19 +748,16 @@
       <c r="D2" t="str">
         <v>Kg</v>
       </c>
-      <c r="E2" t="str">
-        <v>Agro Distributors Ltd</v>
+      <c r="E2">
+        <v>562.5</v>
       </c>
       <c r="F2">
-        <v>562.5</v>
-      </c>
-      <c r="G2">
         <v>25</v>
       </c>
+      <c r="G2" t="str">
+        <v>GHS</v>
+      </c>
       <c r="H2" t="str">
-        <v>GHS</v>
-      </c>
-      <c r="I2" t="str">
         <v>Premium grade sun-dried cocoa beans</v>
       </c>
     </row>
@@ -801,19 +774,16 @@
       <c r="D3" t="str">
         <v>L</v>
       </c>
-      <c r="E3" t="str">
-        <v>West Africa Oils</v>
+      <c r="E3">
+        <v>187.5</v>
       </c>
       <c r="F3">
-        <v>187.5</v>
-      </c>
-      <c r="G3">
         <v>25</v>
       </c>
+      <c r="G3" t="str">
+        <v>GHS</v>
+      </c>
       <c r="H3" t="str">
-        <v>GHS</v>
-      </c>
-      <c r="I3" t="str">
         <v>Refined palm oil for food production</v>
       </c>
     </row>
@@ -830,25 +800,22 @@
       <c r="D4" t="str">
         <v>m</v>
       </c>
-      <c r="E4" t="str">
-        <v>PackRight Ltd</v>
+      <c r="E4">
+        <v>850</v>
       </c>
       <c r="F4">
-        <v>850</v>
-      </c>
-      <c r="G4">
         <v>1</v>
       </c>
+      <c r="G4" t="str">
+        <v>GHS</v>
+      </c>
       <c r="H4" t="str">
-        <v>GHS</v>
-      </c>
-      <c r="I4" t="str">
         <v>100m roll of clear heat-seal packaging film</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>